<commit_message>
Fix bulk upload error handling, dates and required-field checks
Read API errors from their error envelope so duplicates are skipped,
stop day-first parsing from swapping ISO and Excel dates, send
date-time fields as epoch milliseconds, check required built-in fields
in the dry run, and keep one failed request from stopping the upload.
Add vendor columns to the samples and ignore failed_rows.csv.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/notebooks/how_to/inventory/sample_inventory_records.xlsx
+++ b/notebooks/how_to/inventory/sample_inventory_records.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,28 +425,38 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>purpose</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>tiering</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>business_unit</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>is_vendor_model</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>vendor_name</t>
         </is>
       </c>
     </row>
@@ -449,16 +471,20 @@
           <t>Scores retail credit card applications for approval.</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="C2" t="n">
+        <v>1</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>Retail Banking</t>
         </is>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -471,16 +497,20 @@
           <t>Estimates 12-month default probability for small business loans.</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="C3" t="n">
+        <v>1</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
           <t>Commercial Banking</t>
         </is>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -493,16 +523,20 @@
           <t>Forecasts prepayment rates for the residential mortgage book.</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="C4" t="n">
+        <v>2</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
           <t>Retail Banking</t>
         </is>
       </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -515,16 +549,20 @@
           <t>Flags potentially fraudulent card transactions in real time.</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="C5" t="n">
+        <v>1</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
           <t>Retail Banking</t>
         </is>
       </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -537,16 +575,20 @@
           <t>Projects deposit balances for liquidity planning.</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="C6" t="n">
+        <v>2</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -559,16 +601,20 @@
           <t>Predicts which retail customers are likely to close their accounts.</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="C7" t="n">
+        <v>3</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
           <t>Retail Banking</t>
         </is>
       </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -581,16 +627,20 @@
           <t>Ranks overdue accounts by expected recovery.</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="C8" t="n">
+        <v>2</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
           <t>Retail Banking</t>
         </is>
       </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -603,16 +653,20 @@
           <t>Scores transactions for anti-money laundering review.</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="C9" t="n">
+        <v>1</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
           <t>Risk Management</t>
         </is>
       </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -625,16 +679,20 @@
           <t>Measures the impact of rate shocks on net interest income.</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="C10" t="n">
+        <v>1</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -647,14 +705,22 @@
           <t>LLM assistant that drafts replies to customer service queries.</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="C11" t="n">
+        <v>2</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
           <t>Operations</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Example AI Vendor</t>
         </is>
       </c>
     </row>

</xml_diff>